<commit_message>
[+]Se agregan usuarios nuevos
</commit_message>
<xml_diff>
--- a/backend/data/tecnicos.xlsx
+++ b/backend/data/tecnicos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WILMAR\Diagnostico03\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15823B62-E69D-4823-9D7A-AF11BDEAD452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FB5552D-E28F-484C-9BAF-AE7D95E97542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
   <si>
     <t>Cédula</t>
   </si>
@@ -47,6 +47,12 @@
   </si>
   <si>
     <t>Tecnico de Soporte</t>
+  </si>
+  <si>
+    <t>Edgar Albeiro Ramirez Martinez</t>
+  </si>
+  <si>
+    <t>Líder Regional de Soporte</t>
   </si>
 </sst>
 </file>
@@ -97,14 +103,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -444,80 +455,70 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.25" customWidth="1"/>
+    <col min="1" max="1" width="16.25" style="5" customWidth="1"/>
     <col min="2" max="2" width="15.625" customWidth="1"/>
     <col min="3" max="3" width="23.25" customWidth="1"/>
     <col min="4" max="4" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1">
+        <v>123456</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2">
-        <v>123456</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
         <v>1121855145</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="5">
+        <v>88160957</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
[+]Se agregan usuarios con rol, boton de noticias
</commit_message>
<xml_diff>
--- a/backend/data/tecnicos.xlsx
+++ b/backend/data/tecnicos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WILMAR\Diagnostico03\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FB5552D-E28F-484C-9BAF-AE7D95E97542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D057A1B-FFD6-4510-8EE7-FCBB76EB1570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
   <si>
     <t>Cédula</t>
   </si>
@@ -53,6 +53,12 @@
   </si>
   <si>
     <t>Líder Regional de Soporte</t>
+  </si>
+  <si>
+    <t>Rol</t>
+  </si>
+  <si>
+    <t>Tecnico</t>
   </si>
 </sst>
 </file>
@@ -103,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -116,6 +122,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -455,7 +462,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.25" style="5" customWidth="1"/>
@@ -464,7 +471,7 @@
     <col min="4" max="4" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -477,8 +484,11 @@
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -491,8 +501,11 @@
       <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="E2" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1121855145</v>
       </c>
@@ -505,8 +518,11 @@
       <c r="D3" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="E3" s="6" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>88160957</v>
       </c>
@@ -518,6 +534,9 @@
       </c>
       <c r="D4" t="s">
         <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[+] se oculta boton noticias del rol tecnico. Solo visible en rol administrador
</commit_message>
<xml_diff>
--- a/backend/data/tecnicos.xlsx
+++ b/backend/data/tecnicos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WILMAR\Diagnostico03\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D057A1B-FFD6-4510-8EE7-FCBB76EB1570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD875FD2-7638-4C11-B6DB-8896BE3D0626}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -109,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -122,7 +122,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -469,6 +468,7 @@
     <col min="2" max="2" width="15.625" customWidth="1"/>
     <col min="3" max="3" width="23.25" customWidth="1"/>
     <col min="4" max="4" width="19" customWidth="1"/>
+    <col min="5" max="5" width="17.75" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -518,7 +518,7 @@
       <c r="D3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[+] se agregan nuevos usuarios, con opcion de cambio de contraseña y se modfiican logos en header, separando logos del pdf en carpetas distintas
</commit_message>
<xml_diff>
--- a/backend/data/tecnicos.xlsx
+++ b/backend/data/tecnicos.xlsx
@@ -1,87 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WILMAR\Diagnostico03\backend\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD875FD2-7638-4C11-B6DB-8896BE3D0626}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
   <sheets>
     <sheet name="Tecnicos" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
-  <si>
-    <t>Cédula</t>
-  </si>
-  <si>
-    <t>Contraseña</t>
-  </si>
-  <si>
-    <t>Nombre</t>
-  </si>
-  <si>
-    <t>Cargo</t>
-  </si>
-  <si>
-    <t>Administrador</t>
-  </si>
-  <si>
-    <t>Corbeta26*</t>
-  </si>
-  <si>
-    <t>Soporte TI</t>
-  </si>
-  <si>
-    <t>Wilmar Franco</t>
-  </si>
-  <si>
-    <t>Tecnico de Soporte</t>
-  </si>
-  <si>
-    <t>Edgar Albeiro Ramirez Martinez</t>
-  </si>
-  <si>
-    <t>Líder Regional de Soporte</t>
-  </si>
-  <si>
-    <t>Rol</t>
-  </si>
-  <si>
-    <t>Tecnico</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -109,33 +64,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -460,89 +396,472 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="16.25" style="5" customWidth="1"/>
-    <col min="2" max="2" width="15.625" customWidth="1"/>
-    <col min="3" max="3" width="23.25" customWidth="1"/>
-    <col min="4" max="4" width="19" customWidth="1"/>
-    <col min="5" max="5" width="17.75" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E27"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Cédula</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Contraseña</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Nombre</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Cargo</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Rol</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1">
+      <c r="B2">
         <v>123456</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
+      <c r="C2" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Soporte TI</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Administrador</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>88160957</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Corbeta10*</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Edgar Albeiro Ramirez Martinez</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Líder Regional de Soporte</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Administrador</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>80845492</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Corbeta11*</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Erwin Francisco Lis Saldaña</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Coordinador de Soporte TIC</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Administrador</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>1033820304</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Corbeta12*</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Andres Camilo Perez Jimenez</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>1000734283</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Corbeta13*</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Brandon Bleith Marin Cruz</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>79133058</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Corbeta14*</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Carlos Adolfo Lozano Rodriguez</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>11590324</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Corbeta15*</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Carlos Augusto Pineda Roldan</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>80140585</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Corbeta16*</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Cesar Andres Cuevas Carrillo</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>80063906</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Corbeta17*</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Cesar David Mota Serrano</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>1010204069</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Corbeta18*</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Christian German Alonso Segura</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>1233900389</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Corbeta19*</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Cristhian Camilo Villarreal Cortes</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>1033721088</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Corbeta20*</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Daniel Andres Forero Fajardo</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>10301508</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Corbeta21*</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Ever Mauricio Agredo Silva</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>80796479</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Corbeta22*</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Fabian Elias Acosta Fajardo</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>1020760934</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Corbeta23*</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Heyson Nicolas Castiblanco Mora</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>1062304838</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Corbeta24*</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Ivan Camilo Zapata Ospina</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>40437175</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Corbeta25*</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Ivonne Ardila Prada</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>1076624363</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Corbeta26*</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Jairo Alexander Arevalo Salcedo</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>1023932651</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Corbeta27*</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Jairo Suarez Landinez</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>80240931</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Corbeta28*</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Jhon Alexander Barbosa</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>1030667140</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Corbeta29*</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Juan Sebastian Campo Herrera</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>1031131751</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Corbeta30*</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Lisandro Cubillos Reyes</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>1116544966</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Corbeta31*</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Michael Rene Rivas Reyes</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>1022338458</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Corbeta32*</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Oscar Alexander Rodriguez Higuera</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>80056982</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Corbeta33*</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Ricardo Humberto Moreno Melo</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Tecnico</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
         <v>1121855145</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="5">
-        <v>88160957</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" t="s">
-        <v>4</v>
+      <c r="B27" t="str">
+        <v>Corbeta26*</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Wilmar Eulises Franco Beltran</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Tecnico de Soporte</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Tecnico</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D1" numberStoredAsText="1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E27"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>